<commit_message>
docs: board sync (HX1/NU3) + queue NU3 + PUB* specs
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -2620,7 +2620,7 @@
       </c>
       <c r="J34" s="28" t="inlineStr">
         <is>
-          <t>Spec ready — REAL build (not already done): history table exists; add estimated-1RM trend chart + PR cards (heaviest/best e1RM/best volume) + token pass. epley1RM helper + per-session aggregation provided. HX1-Exercise-Detail-Spec.md</t>
+          <t>Built — pending merge/deploy. ExerciseHistory now leads with an Estimated-1RM trend MetricCard (Epley via shared epley1RM; sparkline + DeltaChip + interpretE1rmTrend gated to &gt;=2 sessions) + 3 per-session PR tiles (heaviest set / best e1RM / best volume); chronological table kept. Replaced the naive first-vs-last delta. tsc clean + 29 vitest pass (3 new interpretE1rmTrend cases). Weights kept kg (WK8 useWeightUnit = fast-follow). Visual confirm at post-deploy smoke.</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       </c>
       <c r="J41" s="28" t="inlineStr">
         <is>
-          <t>Spec ready — RE-SCOPED: client already sees adjustment history (expected/actual/deviation + new macros + coach notes). Gap = surface latest applied change as a plain-language banner moment (interpretAdjustment helper) + token pass. NU3-Nutrition-Checkin-Spec.md</t>
+          <t>Spec authored 2026-06-20 → docs/NU3-Nutrition-Checkin-Spec.md (in repo). RE-SCOPED: client already sees adjustment history; gap = surface latest APPLIED adjustment as a 'new target &amp; why' hero banner (interpretAdjustment helper, sign-trap-safe + MacroDistributionRibbon) + CC5 token pass. Implement on clean main AFTER CL2+HX1 merge (shares interpret.ts). Not yet built.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: CL2 + HX1 shipped (merged #166/#167)
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -1499,7 +1499,7 @@
       </c>
       <c r="J11" s="25" t="inlineStr">
         <is>
-          <t>Built — pending merge/deploy. PR-B: WeeklyProgressCard interpretation done. NutritionTargetsCard now CC1/CC2: per-macro % of calories + neutral-tone interpretMacroTargets() line (protein-forward/balanced/carb-led + goal intent), pure fn of stored grams (no BMR/TDEE). tsc clean + 26 vitest pass (incl new interpretMacroTargets cases). Visual confirm at post-deploy smoke.</t>
+          <t>Shipped — merged main PR #166 (ca6e822), deploys to prod via Vercel. WeeklyProgressCard (PR-B) + NutritionTargetsCard now CC1/CC2: per-macro % + interpretMacroTargets() line. Visual confirm at post-deploy smoke.</t>
         </is>
       </c>
     </row>
@@ -2620,7 +2620,7 @@
       </c>
       <c r="J34" s="28" t="inlineStr">
         <is>
-          <t>Built — pending merge/deploy. ExerciseHistory now leads with an Estimated-1RM trend MetricCard (Epley via shared epley1RM; sparkline + DeltaChip + interpretE1rmTrend gated to &gt;=2 sessions) + 3 per-session PR tiles (heaviest set / best e1RM / best volume); chronological table kept. Replaced the naive first-vs-last delta. tsc clean + 29 vitest pass (3 new interpretE1rmTrend cases). Weights kept kg (WK8 useWeightUnit = fast-follow). Visual confirm at post-deploy smoke.</t>
+          <t>Shipped — merged main PR #167 (1b5f9c6), deploys to prod via Vercel. ExerciseHistory leads with Estimated-1RM trend MetricCard (Epley via shared helper; sparkline+delta+interpretE1rmTrend gated &gt;=2 sessions) + 3 per-session PR tiles; chronological table kept. Visual confirm at post-deploy smoke.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: NU3 reopened + re-target spec v2 (orphaned mount found in live smoke)
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -2939,7 +2939,7 @@
       </c>
       <c r="F41" s="13" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="G41" s="17" t="inlineStr">
@@ -2959,7 +2959,7 @@
       </c>
       <c r="J41" s="28" t="inlineStr">
         <is>
-          <t>Shipped — merged main PR #168 (1fb91b0), deploys to prod via Vercel. ClientNutritionAdjustments now leads with a 'Your plan just updated' hero (latest applied adjustment: new kcal + MacroDistributionRibbon + interpretAdjustment 'new target &amp; why' line, sign-trap-safe) + CC5 token pass on history cards. tsc clean + 33 vitest. Visual confirm at post-deploy smoke.</t>
+          <t>RE-TARGET spec ready (v2) — docs/NU3-Nutrition-Checkin-Spec.md. #168 shipped the banner into orphaned ClientNutritionAdjustments.tsx (zero UI effect; caught in live smoke). v2: mount banner in NutritionProgress.tsx (team flow) wired to weekly_progress (calorie_adjustment/new_daily_calories), reuse interpretAdjustment helper (already in interpret.ts), CC5 token pass on per-week Alert, DELETE orphaned component. 1:1 flow out of scope (NutritionPhaseCard already a hero). Live-verify needs a seeded weekly_progress row (table empty pre-launch).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: PUB4 shipped (code-verified, #170); live mobile smoke deferred to launch
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -4043,6 +4043,11 @@
           <t>Mobile landing best practice</t>
         </is>
       </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Shipped (code) — merged main PR #170 (4414be8), live on prod. Mobile sticky CTA bar (single-source primaryCta + IntersectionObserver, md:hidden, safe-area pb) + hero LCP &lt;link rel=preload as=image&gt;. tsc + build clean, faithful diff. LIVE MOBILE SMOKE NOT YET DONE: landing '/' is unreachable in waitlist mode (anon -&gt; /waitlist, logged-in -&gt; /dashboard) + Chrome resize didn't give a true &lt;=767px viewport. Self-verifies at launch (waitlist off); or add a mocked-logged_out component test for durable coverage.</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="42" customHeight="1">
       <c r="A65" s="15" t="inlineStr">

</xml_diff>

<commit_message>
docs: PUB9 shipped + live-verified (#171)
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -4283,6 +4283,11 @@
           <t>Standard pattern</t>
         </is>
       </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>Shipped + LIVE-VERIFIED — merged main PR #171 (5da0522), on prod. og:image/twitter:image now ABSOLUTE https://theigu.com/og-image.png (was relative -&gt; broke scraper previews) + width/height/alt/locale; Organization enriched (square logo, areaServed Kuwait, contactPoint) + ProfessionalService Kuwait node (no prices, pending level-pricing). Verified live via served-HTML head fetch; both JSON-LD blocks schema-valid (0 err). OG image already on-brand (IGU wordmark, 2400x1260). NOTE: CMS social_links all empty -&gt; footer shows no socials + sameAs omitted (content to-do).</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="42" customHeight="1">
       <c r="A70" s="11" t="inlineStr">

</xml_diff>

<commit_message>
docs: WA1 spec (coach WhatsApp session button) + board row
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -946,7 +946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J88"/>
+  <dimension ref="A1:J89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5269,6 +5269,58 @@
       <c r="J88" s="24" t="inlineStr">
         <is>
           <t>Resolved — NOT a real bug. Stale cached dev bundle on the phone (long session: many HMR reloads + 2 LAN-IP changes + mirror reconnects) -&gt; module load failure -&gt; error boundary (same family as the SPA stale-chunk pattern). Disproven: CC faithful DB rebuild of the payment-exempt-sub shape + activity data rendered CLEAN in both Playwright Chromium AND real WebKit; and prod theigu.com/coach renders perfectly with the same real coach data. Dev-session artifact, not prod.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>WA1</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Messaging</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Workout completion</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Add a "Message coach about this session" WhatsApp deep-link on the 1:1 workout completion sheet, pre-filled with the WK7 session recap (volume/sets/time/new PRs).</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Flagship of the hybrid messaging direction; WhatsApp is the preferred client&lt;-&gt;coach channel in-region; reuses existing WK7 summary + coach whatsapp_number.</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>WorkoutCompletionSheet.tsx, WorkoutSessionV2.tsx, + get_coach_whatsapp_for_client RPC migration</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Ladder/Future coach contact</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Spec ready — docs/WA1-coach-whatsapp-session-button.md (2026-06-20). Needs new gated RPC (whatsapp not in get_coach_for_client) + sheet button + 1:1 service gate. Hybrid decision confirmed; in-app care-team messaging stays.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: PUB2 shipped + live-verified (#174)
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -3949,6 +3949,11 @@
           <t>SaaS pricing pages (Mobbin Sites)</t>
         </is>
       </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Shipped + LIVE-VERIFIED -- merged main PR #174 (4f28d97), on prod. Services pricing clarity: 'Most popular' badge + ring/scale emphasis on the Hybrid card (slug-matched via service.slug=='hybrid', not name), tightened per-card CTAs (Join the team / Start online / Start hybrid / Start in-person via CTA_BY_SLUG), and the team start-date announcement block surfaced on Services (mirrors Index; loadTeamPlanSettings switched to .maybeSingle()). ComparisonTable untouched. Verified live on theigu.com/services after a hard-reload past a stale apex cache: Hybrid badge + emphasis, 4 tightened CTAs, prices 10/30/95/145, announcement renders ('Next team program starts soon!'; next_program_start_date null so the date sub-line is not exercised). tsc+build clean per CC. Note: PUB2 also pre-existed inside the Capacitor Phase-1 commit; de-duped during the feat/capacitor-mobile detangle (now main-only).</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="42" customHeight="1">
       <c r="A63" s="15" t="inlineStr">

</xml_diff>

<commit_message>
docs: PUB1 shipped (code + deploy-verified); live anon smoke deferred (waitlist on) (#175)
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -3902,6 +3902,11 @@
           <t>Future / WHOOP marketing sites (Mobbin Sites)</t>
         </is>
       </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Shipped (code) + deploy-verified -- merged main PR #175 (6d530c6), live on prod. Hero social-proof strip (new HeroSocialProof.tsx, sibling right after heroCtaRef so PUB4's IntersectionObserver bounds are untouched): founding-cohort pill (Star icon; FOUNDING_DEFAULT shown by default; CMS-overridable via homepage/social_proof.founding_line; hideable via founding_enabled='false') + a dormant 3-cell stats row where each cell renders only when its stat{n}_value is set; component returns null when nothing to show. No live DB read (pre-launch numbers are 1 coach/0 testimonials/0 paying -- numbers come only from CMS values). tsc+build clean, diff matches spec exactly. LIVE ANON SMOKE DEFERRED: landing '/' is unreachable while waitlist is ON (anon -&gt; /waitlist, logged-in -&gt; role home) -- confirmed via the main vercel.app alias redirecting anon to /waitlist. Self-verifies at launch (waitlist off); or preview now by toggling waitlist off in an incognito window. Content to-do (Hasan): founding line is live by default; populate homepage/social_proof stat rows in admin as real numbers/testimonials arrive (keys in docs/PUB1-Hero-Social-Proof-Spec.md).</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="42" customHeight="1">
       <c r="A62" s="11" t="inlineStr">

</xml_diff>

<commit_message>
docs: PUB3 shipped (code + deploy-verified); visual smoke noted (#176)
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -4006,6 +4006,11 @@
           <t>Future / Centr coach bios</t>
         </is>
       </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Shipped (code) + deploy-verified -- merged main PR #176 (450a458), live on prod (production aliases theigu.com + www point to this deploy, state READY). MeetOurTeam coach cards now surface a 'Certifications' block (Award icon + first 2 qualifications as outline badges with truncate+title, plus '+N more') ABOVE specializations, gated on coach.qualifications presence -- certs that were dialog-only are now on the card. Lead styling / short_bio / specializations / CoachDetailDialog left untouched; free-text quals rendered directly (no getLabel). tsc+build clean; diff matches spec exactly. LIVE VISUAL SMOKE INCOMPLETE: /meet-our-team rendered but the Chrome automation could not snapshot it (page never reached document_idle -- open connections/hanging request in the admin session); this is a pure conditional render of already-fetched data, low risk -- re-eyeball via an authenticated session at leisure. Content (Hasan): lead coach has 9 quals populated (card shows MB BCh BAO (Hons) / ACE-CPT / +7 more), but short_bio (the philosophy/standout line) is empty -- populate a 1-2 sentence standout per coach.</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="42" customHeight="1">
       <c r="A64" s="11" t="inlineStr">

</xml_diff>

<commit_message>
docs: CL1 shipped (code); client-session visual smoke pending (#178)
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -1450,6 +1450,11 @@
           <t>Future / Oura home</t>
         </is>
       </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Shipped (code) -- merged main PR #178 (0f1b7b6), auto-deploys to prod via Vercel. Restructured the ACTIVE client dashboard overview in NewClientOverview.tsx (the live surface; the card-grid OverviewSection inside ClientDashboardLayout is orphaned dead code -- left untouched). New order: interrupts (PaymentAttentionBanner/AlertsCard) -&gt; one hero (TodaysWorkoutHero, with the programCount=0 'coach is preparing your program' empty-state preserved) -&gt; LogTodayCard -&gt; single-column ranked stack (NutritionTargets -&gt; WeeklyProgress -&gt; Adherence -&gt; Coach -&gt; CareTeam) -&gt; QuickActionsGrid -&gt; quiet 'Account' group (border-t + muted heading wrapping PlanBillingCard only). Both 2-col grids dropped; billing demoted; all 11 cards present exactly once with props/hooks/loadDashboardData/skeleton/empty-state unchanged (reorder only). tsc+build clean; diff matches spec. LIVE VISUAL SMOKE PENDING: /dashboard is auth-gated to an active client (admin/coach are redirected) so it is NOT reachable through the admin session -- verify the mobile single-column read, desktop-not-broken, and empty-state hero-swap via a test-client login or the Capacitor build. Client nutrition PAGE intentionally untouched (separate NU* items own it).</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="15" t="inlineStr">

</xml_diff>

<commit_message>
docs: NU8 Phase 1 (team nutrition consolidation) shipped + live (#179); Phase 2 pending
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -946,7 +946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J89"/>
+  <dimension ref="A1:J90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5341,6 +5341,58 @@
       <c r="J89" t="inlineStr">
         <is>
           <t>Shipped (code + RPC verified) — merged main PR #173 (b188445), live on prod. get_coach_whatsapp_for_client RPC registered (20260621120000 via migration repair+db push), SECURITY DEFINER, EXECUTE to authenticated/service_role only (anon denied). 'Message coach about this session' button on 1:1 workout-completion sheet (mobile+desktop), wa.me deep-link pre-filled from WK7 summary; team_plan excluded; separate ref-guarded fetch (not in loadSession burst). tsc+build clean. LIVE VISUAL smoke pending a 1:1 client + coach whatsapp_number set (team session won't show it by design). Bonus: 7 drifted WK8/WK9 migrations (20260619*) reconciled into schema_migrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>NU8</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Nutrition (Team + 1:1)</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Consolidate the client nutrition pages into one scroll: remove the Goal Setting/Progress Tracker top tabs AND the nested Progress/Graphs tabs; targets hero with an Edit-targets sheet, inline trend (range + Weight/Body-fat toggle), weekly check-ins. Unify team + 1:1.</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Removes 3-layer redundant tab nesting; information scent; Mobbin-grounded.</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>TeamNutrition.tsx, NutritionProgress.tsx, NutritionGoal.tsx, ClientNutrition.tsx</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>MacroFactor / Lifesum / Yazio / Alma / MyFitnessPal (ios)</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Phase 1 (team) SHIPPED + LIVE (deploy-verified) -- merged main PR #179 (7f8e92b); production aliases (theigu.com/www) point to it, READY. TeamNutrition consolidated to one scroll: top-level Goal/Progress tabs + nested Progress/Graphs tabs removed. Hero gained MacroDistributionRibbon + an 'Edit targets' responsive sheet (mobile vaul Drawer repositionInputs=false per BUG6 + DrawerScrollArea; desktop Dialog + DialogScrollArea) hosting NutritionGoal(onSaved=close+refresh) -- replaces the navigate-away 'Change Goal'. Inline trend = 4W/12W/All range pills + Weight|Body-fat toggle (weeklyProgress filtered upstream; graph internals untouched); WeekCard list unchanged; no-goal empty state opens the sheet. NutritionGoal gained optional onSaved prop (non-breaking). tsc+build+eslint clean; diff matches spec. TEST-CLIENT VISUAL PENDING (auth-gated to active team client; admin/coach redirected) -- verify sheet save-&gt;close-&gt;refresh, trend range/toggle, and mobile keyboard via a team test-client login / Capacitor. FOLLOW-UPS (minor, non-blocking): (1) stray ?tab= links in QuickActionsGrid/AlertsCard now no-op -- tidy; (2) loadData's 'No Active Goal' destructive toast fires on the first-time no-goal path next to the 'Set your targets' empty state -- misleading, soften/remove. PHASE 2 (1:1 ClientNutrition alignment) PENDING -- separate branch/PR per docs/NU-Client-Nutrition-Redesign-Spec.md.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: CL1 + NU8 Phase 1 live-verified via team client (#178, #179)
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -1452,7 +1452,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Shipped (code) -- merged main PR #178 (0f1b7b6), auto-deploys to prod via Vercel. Restructured the ACTIVE client dashboard overview in NewClientOverview.tsx (the live surface; the card-grid OverviewSection inside ClientDashboardLayout is orphaned dead code -- left untouched). New order: interrupts (PaymentAttentionBanner/AlertsCard) -&gt; one hero (TodaysWorkoutHero, with the programCount=0 'coach is preparing your program' empty-state preserved) -&gt; LogTodayCard -&gt; single-column ranked stack (NutritionTargets -&gt; WeeklyProgress -&gt; Adherence -&gt; Coach -&gt; CareTeam) -&gt; QuickActionsGrid -&gt; quiet 'Account' group (border-t + muted heading wrapping PlanBillingCard only). Both 2-col grids dropped; billing demoted; all 11 cards present exactly once with props/hooks/loadDashboardData/skeleton/empty-state unchanged (reorder only). tsc+build clean; diff matches spec. LIVE VISUAL SMOKE PENDING: /dashboard is auth-gated to an active client (admin/coach are redirected) so it is NOT reachable through the admin session -- verify the mobile single-column read, desktop-not-broken, and empty-state hero-swap via a test-client login or the Capacitor build. Client nutrition PAGE intentionally untouched (separate NU* items own it).</t>
+          <t>Shipped + LIVE-VERIFIED (2026-06-23) -- merged main PR #178 (0f1b7b6), live on prod. Restructured the ACTIVE client dashboard overview in NewClientOverview.tsx (the card-grid OverviewSection in ClientDashboardLayout is orphaned dead code, untouched). Verified live via a team client (Hasan, desktop, /dashboard): interrupts (AlertsCard 'Missing Weight Logs') -&gt; Today's Workout hero -&gt; single-column ranked stack (Daily Targets -&gt; This Week -&gt; Adherence -&gt; Your Coach -&gt; My Care Team) -&gt; QuickActionsGrid (Weekly Check-In / Nutrition / Exercise Library) -&gt; quiet 'Account' group (border-t + muted heading) with PlanBillingCard demoted to the bottom. Both 2-col grids gone; all cards present once. tsc+build clean. Mobile reads the same single column (grids dropped); explicit phone pass optional.</t>
         </is>
       </c>
     </row>
@@ -4013,7 +4013,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>Shipped (code) + deploy-verified -- merged main PR #176 (450a458), live on prod (production aliases theigu.com + www point to this deploy, state READY). MeetOurTeam coach cards now surface a 'Certifications' block (Award icon + first 2 qualifications as outline badges with truncate+title, plus '+N more') ABOVE specializations, gated on coach.qualifications presence -- certs that were dialog-only are now on the card. Lead styling / short_bio / specializations / CoachDetailDialog left untouched; free-text quals rendered directly (no getLabel). tsc+build clean; diff matches spec exactly. LIVE VISUAL SMOKE INCOMPLETE: /meet-our-team rendered but the Chrome automation could not snapshot it (page never reached document_idle -- open connections/hanging request in the admin session); this is a pure conditional render of already-fetched data, low risk -- re-eyeball via an authenticated session at leisure. Content (Hasan): lead coach has 9 quals populated (card shows MB BCh BAO (Hons) / ACE-CPT / +7 more), but short_bio (the philosophy/standout line) is empty -- populate a 1-2 sentence standout per coach.</t>
+          <t>Shipped + LIVE-VERIFIED (2026-06-23) -- merged main PR #176 (450a458), live on prod. MeetOurTeam coach cards now surface a 'Certifications' block (Award icon + first 2 qualifications as outline badges + '+N more') ABOVE Specializations, gated on coach.qualifications. Verified live on theigu.com/meet-our-team (authenticated client session): lead coach (Hasan Dashti, Lead badge + red ring) shows Certifications = 'MB BCh BAO (Hons)' / 'ACE-CPT' / '+7 more', then Specializations (General Fitness/Strength Training/Bodybuilding/+6 more). Lead styling / CoachDetailDialog / specializations untouched; free-text quals rendered directly (no getLabel). tsc+build clean; diff matches spec. CONTENT (Hasan): lead coach short_bio (the philosophy/standout line) is still empty -- card shows no standout line; populate a 1-2 sentence standout per coach.</t>
         </is>
       </c>
     </row>
@@ -5392,7 +5392,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>Phase 1 (team) SHIPPED + LIVE (deploy-verified) -- merged main PR #179 (7f8e92b); production aliases (theigu.com/www) point to it, READY. TeamNutrition consolidated to one scroll: top-level Goal/Progress tabs + nested Progress/Graphs tabs removed. Hero gained MacroDistributionRibbon + an 'Edit targets' responsive sheet (mobile vaul Drawer repositionInputs=false per BUG6 + DrawerScrollArea; desktop Dialog + DialogScrollArea) hosting NutritionGoal(onSaved=close+refresh) -- replaces the navigate-away 'Change Goal'. Inline trend = 4W/12W/All range pills + Weight|Body-fat toggle (weeklyProgress filtered upstream; graph internals untouched); WeekCard list unchanged; no-goal empty state opens the sheet. NutritionGoal gained optional onSaved prop (non-breaking). tsc+build+eslint clean; diff matches spec. TEST-CLIENT VISUAL PENDING (auth-gated to active team client; admin/coach redirected) -- verify sheet save-&gt;close-&gt;refresh, trend range/toggle, and mobile keyboard via a team test-client login / Capacitor. FOLLOW-UPS (minor, non-blocking): (1) stray ?tab= links in QuickActionsGrid/AlertsCard now no-op -- tidy; (2) loadData's 'No Active Goal' destructive toast fires on the first-time no-goal path next to the 'Set your targets' empty state -- misleading, soften/remove. PHASE 2 (1:1 ClientNutrition alignment) PENDING -- separate branch/PR per docs/NU-Client-Nutrition-Redesign-Spec.md.</t>
+          <t>Phase 1 (team) SHIPPED + LIVE-VERIFIED (2026-06-23) -- merged main PR #179 (7f8e92b), live on prod. Verified live via a team client (Hasan, desktop, /nutrition-team): one scroll, NO tabs (Goal/Progress + nested Progress/Graphs both removed), new subtitle. Hero = Fat Loss Phase, Current Targets 1751 kcal + MacroDistributionRibbon (P138/F78/C124, red/amber/blue) + 'Edit targets'. Edit targets opens the responsive sheet (desktop Dialog) hosting the NutritionGoal editor (donut + targets + journey + its own Change Goal) in-context with no navigation, closes cleanly. Trend block: 4W/12W/All range pills + Weight|Body-fat toggle (toggle swaps the graph live); Weekly Logs WeekCard expanded with the full check-in form. NutritionGoal gained optional onSaved. tsc+build+eslint clean. REMAINING: mobile Drawer + keyboard (repositionInputs=false) still needs a phone/Capacitor pass; the save-&gt;deactivate+insert goal cycle was NOT triggered live (would mutate the test client's goal). FOLLOW-UPS (minor): (1) stray ?tab= links in QuickActionsGrid/AlertsCard now no-op -- tidy; (2) loadData 'No Active Goal' destructive toast on the first-time no-goal path -- soften. PHASE 2 (1:1 ClientNutrition alignment) PENDING -- separate branch/PR per docs/NU-Client-Nutrition-Redesign-Spec.md.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: RO Phase 1 shipped + live-verified (RO2/RO3, #181); Phase 2 RPC pending
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -2143,6 +2143,11 @@
           <t>Superhuman / Front list rows</t>
         </is>
       </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Phase 1 SHIPPED + LIVE-VERIFIED (2026-06-23) -- merged main PR #181 (a604aea), live on prod. Coach My Clients roster redesigned (CoachMyClientsPage.tsx): needs-attention strip on top (jump chips from get_coach_roster_attention tiles/client_ids + awaitingPayment count; zero-count muted) + ACTIVE-FIRST reorder (action sections moved below, collapse-when-empty) + scannable two-line row (rail · name · plan / status · adherence · check-ins · last weigh-in, sm:grid-cols-4 aligned columns) + consolidated alert cluster (check-in-overdue / payment / adjustment from client_ids + unread + deload; icons only when flagged). Verified live via coach test session (4 wired test clients): strip shows '1 check-ins overdue · 9d' (seeded +hybrid quiet client) and that row shows the Clock alert icon; active roster leads; aligned columns render. tsc+build+eslint clean. PHASE 1 LIMITATION (RLS, confirmed live): the row's 'Last weigh-in' reads weight_logs CLIENT-SIDE, which coach RLS hides, so it shows 'No check-in' for ALL rows (even +online which has 9 logs). The strip's overdue count is correct because it comes from the SECURITY DEFINER RPC. =&gt; PHASE 2 RPC must feed last-weigh-in + adherence + check-ins X/3 (not just adherence). PHASE 2 PENDING: get_coach_roster_stats() / useCoachRosterStats() for adherence % + weekly check-ins + no-program alert + adherence sort -- own branch/PR per docs/RO-Coach-Roster-Redesign-Spec.md.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="42" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
@@ -2188,6 +2193,11 @@
       <c r="I25" s="16" t="inlineStr">
         <is>
           <t>CRM inboxes</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>SHIPPED (RO Phase 1, PR #181 a604aea, live + verified 2026-06-23) -- added 'Check-in due' sort (days_since_check_in desc, nulls last) alongside At-risk-first + Name, beside the existing search + plan filter. Adherence sort deferred to RO Phase 2 (needs the stats RPC).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: CO6 + RO Phase 2 shipped & live-verified (#183, #182); coach-RLS weigh-in follow-up noted
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -1950,6 +1950,11 @@
           <t>Intercom Inbox</t>
         </is>
       </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Shipped + LIVE-VERIFIED (2026-06-23) -- merged main PR #183 (57e7720), live on prod. Coach client view is now a MASTER-DETAIL workspace inside the coach shell (new CoachClientsWorkspace): the CoachSidebar global nav is preserved (no more dead-end page), a persistent compact roster on the left (reuses the roster hooks -- name + plan + adherence/check-ins + alert dots + urgency rail, search + sort, 'Full queue' -&gt; ?view=queue keeps Pending/At-Risk/approvals reachable), and the selected client's detail (ClientOverviewPanel, extracted from the now-deleted standalone CoachClientOverview) in the right pane. App.tsx repoints /coach/clients/:id into CoachDashboard (shell); CoachDashboard derives section from the path. Verified live via coach session (desktop): clicking a client swaps the RIGHT PANE CLIENT-SIDE (no reload), master stays, row highlights, sidebar persists, the 8 section tabs work; 'Select a client' empty state when none selected; check-ins X/3 + tone + alert dots populate from the RO Phase 2 RPC. tsc+build+eslint clean. KNOWN FOLLOW-UP (separate ticket): the detail's Overview 'Last weigh-in' card + Nutrition trend still read weight_logs client-side (coach RLS) -&gt; 'No weigh-ins yet' even with logs; needs a coach-scoped read like get_coach_roster_stats. MOBILE pending a phone pass (drawer master + the two 'Clients' buttons + lg pane-height calc(100vh-12rem) nudge). Pairs with CO7 (per-tab accordion) if desired -- separate.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="42" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
@@ -2145,7 +2150,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Phase 1 SHIPPED + LIVE-VERIFIED (2026-06-23) -- merged main PR #181 (a604aea), live on prod. Coach My Clients roster redesigned (CoachMyClientsPage.tsx): needs-attention strip on top (jump chips from get_coach_roster_attention tiles/client_ids + awaitingPayment count; zero-count muted) + ACTIVE-FIRST reorder (action sections moved below, collapse-when-empty) + scannable two-line row (rail · name · plan / status · adherence · check-ins · last weigh-in, sm:grid-cols-4 aligned columns) + consolidated alert cluster (check-in-overdue / payment / adjustment from client_ids + unread + deload; icons only when flagged). Verified live via coach test session (4 wired test clients): strip shows '1 check-ins overdue · 9d' (seeded +hybrid quiet client) and that row shows the Clock alert icon; active roster leads; aligned columns render. tsc+build+eslint clean. PHASE 1 LIMITATION (RLS, confirmed live): the row's 'Last weigh-in' reads weight_logs CLIENT-SIDE, which coach RLS hides, so it shows 'No check-in' for ALL rows (even +online which has 9 logs). The strip's overdue count is correct because it comes from the SECURITY DEFINER RPC. =&gt; PHASE 2 RPC must feed last-weigh-in + adherence + check-ins X/3 (not just adherence). PHASE 2 PENDING: get_coach_roster_stats() / useCoachRosterStats() for adherence % + weekly check-ins + no-program alert + adherence sort -- own branch/PR per docs/RO-Coach-Roster-Redesign-Spec.md.</t>
+          <t>Phase 1 SHIPPED + LIVE-VERIFIED (2026-06-23) -- merged main PR #181 (a604aea), live on prod. Coach My Clients roster redesigned (CoachMyClientsPage.tsx): needs-attention strip on top (jump chips from get_coach_roster_attention tiles/client_ids + awaitingPayment count; zero-count muted) + ACTIVE-FIRST reorder (action sections moved below, collapse-when-empty) + scannable two-line row (rail · name · plan / status · adherence · check-ins · last weigh-in, sm:grid-cols-4 aligned columns) + consolidated alert cluster (check-in-overdue / payment / adjustment from client_ids + unread + deload; icons only when flagged). Verified live via coach test session (4 wired test clients): strip shows '1 check-ins overdue · 9d' (seeded +hybrid quiet client) and that row shows the Clock alert icon; active roster leads; aligned columns render. tsc+build+eslint clean. PHASE 1 LIMITATION (RLS, confirmed live): the row's 'Last weigh-in' reads weight_logs CLIENT-SIDE, which coach RLS hides, so it shows 'No check-in' for ALL rows (even +online which has 9 logs). The strip's overdue count is correct because it comes from the SECURITY DEFINER RPC. =&gt; PHASE 2 RPC must feed last-weigh-in + adherence + check-ins X/3 (not just adherence). PHASE 2 PENDING: get_coach_roster_stats() / useCoachRosterStats() for adherence % + weekly check-ins + no-program alert + adherence sort -- own branch/PR per docs/RO-Coach-Roster-Redesign-Spec.md. || PHASE 2 LIVE-VERIFIED (2026-06-23): get_coach_roster_stats() applied to prod (RO Phase 2 PR #182 frontend merged; function applied via MCP raw SQL -- SECURITY DEFINER, anon revoked, authenticated granted; a later supabase db push registers the merged migration cleanly). Roster + the CO6 master now show real check-ins X/3 + RPC-fed last-weigh-in (fixes the Phase-1 RLS 'No check-in') + no-program/alert dots; adherence shows '--' until adherence_logs/weekly_progress adherence data exists for these clients. Confirmed live in the coach session.</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2202,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>SHIPPED (RO Phase 1, PR #181 a604aea, live + verified 2026-06-23) -- added 'Check-in due' sort (days_since_check_in desc, nulls last) alongside At-risk-first + Name, beside the existing search + plan filter. Adherence sort deferred to RO Phase 2 (needs the stats RPC).</t>
+          <t>SHIPPED (RO Phase 1, PR #181 a604aea, live + verified 2026-06-23) -- added 'Check-in due' sort (days_since_check_in desc, nulls last) alongside At-risk-first + Name, beside the existing search + plan filter. Adherence sort deferred to RO Phase 2 (needs the stats RPC). Adherence sort now ACTIVE (RO Phase 2 live).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
board: add SE1 (Sessions+booking), WK10 (Workouts calendar), GC1 (GCal future); track CO6/RO specs
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -946,7 +946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J90"/>
+  <dimension ref="A1:J93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5408,6 +5408,162 @@
       <c r="J90" t="inlineStr">
         <is>
           <t>BOTH PHASES SHIPPED + LIVE-VERIFIED (2026-06-23). Client nutrition consolidated to one scroll, zero tabs, team + 1:1 sharing the shape (hero -&gt; log -&gt; trend -&gt; weekly input). PHASE 1 (team, PR #179 7f8e92b): /nutrition-team verified live via a team client -- no tabs, hero + macro ribbon + 'Edit targets' Dialog hosting the goal editor in-context, 4W/12W/All range + Weight|Body-fat toggle, WeekCard check-ins. PHASE 2 (1:1, PR #180 69c9729): /nutrition-client verified live via a seeded 1:1-Online test client -- NutritionPhaseCard hero (read-only, 'On Track', 2100 kcal + ribbon, expected vs actual rate strip computed from seeded weight logs) + 'Message coach to adjust' link + weekly ribbon + inline Log Today + trend (range/toggle on real seeded data, weight line vs target) + 'This week' ClientNutritionProgress form. No tabs. NutritionGoal gained optional onSaved. tsc+build+eslint clean on both. TEST ACCOUNTS (payment-exempt, +alias emails): Team / 1:1 Online / 1:1 Hybrid / 1:1 In-Person created by Hasan; 3 1:1 accounts seeded with active nutrition_phases (Summer Cut / Lean Bulk / Fat Loss Phase) + 9 weight_logs on Online -- retained for ongoing feature testing. REMAINING: mobile Drawer + keyboard (NU Phase 1 Edit-targets sheet, repositionInputs=false) still needs a phone/Capacitor pass. FOLLOW-UPS (minor): stray ?tab= links in QuickActionsGrid/AlertsCard now no-op; loadData 'No Active Goal' destructive toast on first-time no-goal path -- soften.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="11" t="inlineStr">
+        <is>
+          <t>SE1</t>
+        </is>
+      </c>
+      <c r="B91" s="12" t="inlineStr">
+        <is>
+          <t>Sessions</t>
+        </is>
+      </c>
+      <c r="C91" s="12" t="inlineStr">
+        <is>
+          <t>Coach SessionsTab + client /sessions</t>
+        </is>
+      </c>
+      <c r="D91" s="12" t="inlineStr">
+        <is>
+          <t>Redesign to grouped Upcoming/Past lists (date chips + status pills) both sides; then request-&gt;confirm booking (client requests status=requested -&gt; coach confirms/declines); availability slots later phase</t>
+        </is>
+      </c>
+      <c r="E91" s="12" t="inlineStr">
+        <is>
+          <t>Sessions surface is a bare ad-hoc digest; both coach+client need to book; clean Sessions(appointments) vs Workouts(training) boundary</t>
+        </is>
+      </c>
+      <c r="F91" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G91" s="14" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H91" s="12" t="inlineStr">
+        <is>
+          <t>client-overview/tabs/SessionsTab.tsx, pages/sessions, direct_calendar_sessions</t>
+        </is>
+      </c>
+      <c r="I91" s="12" t="inlineStr">
+        <is>
+          <t>Calendly / Cal.com booking; Practo appointments</t>
+        </is>
+      </c>
+      <c r="J91" s="24" t="inlineStr">
+        <is>
+          <t>Spec ready - docs/SE-Sessions-Tab-Booking-Spec.md (CC handoff)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="11" t="inlineStr">
+        <is>
+          <t>WK10</t>
+        </is>
+      </c>
+      <c r="B92" s="12" t="inlineStr">
+        <is>
+          <t>Workout</t>
+        </is>
+      </c>
+      <c r="C92" s="12" t="inlineStr">
+        <is>
+          <t>Coach client Workouts tab</t>
+        </is>
+      </c>
+      <c r="D92" s="12" t="inlineStr">
+        <is>
+          <t>Calendar-forward week grid + per-day +menu (Blank / Saved / Assign program in-context / Create program scoped to client) + Program history strip; reuse DirectClientCalendar/AssignFromLibraryDialog/ClientProgramList</t>
+        </is>
+      </c>
+      <c r="E92" s="12" t="inlineStr">
+        <is>
+          <t>Today Assign navigates away + calendar hidden in a Sheet; no at-a-glance week; building custom program abandons the client page</t>
+        </is>
+      </c>
+      <c r="F92" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G92" s="14" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H92" s="12" t="inlineStr">
+        <is>
+          <t>client-overview/tabs/WorkoutsTab.tsx, coach/programs/*</t>
+        </is>
+      </c>
+      <c r="I92" s="12" t="inlineStr">
+        <is>
+          <t>TrueCoach calendar; Runna day-list</t>
+        </is>
+      </c>
+      <c r="J92" s="24" t="inlineStr">
+        <is>
+          <t>Spec ready - docs/WK-Coach-Workouts-Calendar-Spec.md (CC handoff)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="11" t="inlineStr">
+        <is>
+          <t>GC1</t>
+        </is>
+      </c>
+      <c r="B93" s="12" t="inlineStr">
+        <is>
+          <t>Sessions</t>
+        </is>
+      </c>
+      <c r="C93" s="12" t="inlineStr">
+        <is>
+          <t>Coach + client</t>
+        </is>
+      </c>
+      <c r="D93" s="12" t="inlineStr">
+        <is>
+          <t>Google Calendar 2-way sync of booked sessions (OAuth + Calendar API + token storage/refresh; reminders; later read busy-times). Must work inside Capacitor WebView for native.</t>
+        </is>
+      </c>
+      <c r="E93" s="12" t="inlineStr">
+        <is>
+          <t>Sessions land in the personal calendars both sides actually live in; reduces no-shows</t>
+        </is>
+      </c>
+      <c r="F93" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G93" s="14" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="H93" s="12" t="inlineStr">
+        <is>
+          <t>new edge fns + token table; direct_calendar_sessions</t>
+        </is>
+      </c>
+      <c r="I93" s="12" t="inlineStr">
+        <is>
+          <t>Calendly GCal connect</t>
+        </is>
+      </c>
+      <c r="J93" s="24" t="inlineStr">
+        <is>
+          <t>Future phase - after Sessions booking (Phase 2) ships. Captured; not started</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
board: Progress (PR1), Care Team (CT1), Profile (PF1) tab redesign specs + mocks
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -946,7 +946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J93"/>
+  <dimension ref="A1:J96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5564,6 +5564,162 @@
       <c r="J93" s="24" t="inlineStr">
         <is>
           <t>Future phase - after Sessions booking (Phase 2) ships. Captured; not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="11" t="inlineStr">
+        <is>
+          <t>PR1</t>
+        </is>
+      </c>
+      <c r="B94" s="12" t="inlineStr">
+        <is>
+          <t>Progress</t>
+        </is>
+      </c>
+      <c r="C94" s="12" t="inlineStr">
+        <is>
+          <t>Coach client Progress tab</t>
+        </is>
+      </c>
+      <c r="D94" s="12" t="inlineStr">
+        <is>
+          <t>Add CC1 metric-card summary row (weight/body-fat/volume + deltas + sparklines) + status header above the existing weight-trend hero; two-up Measurements + Volume below. Display-only regroup of CoachNutritionGraphs + VolumeChart</t>
+        </is>
+      </c>
+      <c r="E94" s="12" t="inlineStr">
+        <is>
+          <t>Raw chart dump today; the numbers a coach scans first arent surfaced; no shared visual language</t>
+        </is>
+      </c>
+      <c r="F94" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G94" s="14" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H94" s="12" t="inlineStr">
+        <is>
+          <t>client-overview/tabs/ProgressTab.tsx, CoachNutritionGraphs, VolumeChart</t>
+        </is>
+      </c>
+      <c r="I94" s="12" t="inlineStr">
+        <is>
+          <t>Oura/WHOOP insights; CC1 metric card</t>
+        </is>
+      </c>
+      <c r="J94" s="24" t="inlineStr">
+        <is>
+          <t>Spec + mock ready - docs/PR-Progress-Tab-Redesign-Spec.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="11" t="inlineStr">
+        <is>
+          <t>CT1</t>
+        </is>
+      </c>
+      <c r="B95" s="12" t="inlineStr">
+        <is>
+          <t>Care Team</t>
+        </is>
+      </c>
+      <c r="C95" s="12" t="inlineStr">
+        <is>
+          <t>CareTeamCard + CareTeamMessagesPanel</t>
+        </is>
+      </c>
+      <c r="D95" s="12" t="inlineStr">
+        <is>
+          <t>Polish roster to role-coloured chips (coach/dietitian/physio) + staff-only banner; restyle team thread to own-vs-other bubbles w/ mentions. Presentation pass, no schema/RLS change</t>
+        </is>
+      </c>
+      <c r="E95" s="12" t="inlineStr">
+        <is>
+          <t>Components predate the current card/chip/thread language; read as a flat list + log</t>
+        </is>
+      </c>
+      <c r="F95" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G95" s="14" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H95" s="12" t="inlineStr">
+        <is>
+          <t>coach/CareTeamCard.tsx, nutrition/CareTeamMessagesPanel.tsx</t>
+        </is>
+      </c>
+      <c r="I95" s="12" t="inlineStr">
+        <is>
+          <t>Slack threads; clinical care-team UIs</t>
+        </is>
+      </c>
+      <c r="J95" s="24" t="inlineStr">
+        <is>
+          <t>Spec + mock ready - docs/CT-CareTeam-Tab-Redesign-Spec.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="11" t="inlineStr">
+        <is>
+          <t>PF1</t>
+        </is>
+      </c>
+      <c r="B96" s="12" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="C96" s="12" t="inlineStr">
+        <is>
+          <t>Coach client Profile tab</t>
+        </is>
+      </c>
+      <c r="D96" s="12" t="inlineStr">
+        <is>
+          <t>Add identity header card (avatar+name+plan+status pill); swap shadcn Badges for the standard rounded status pills; auto-fit the demographics grid. Light polish, already well-built, read-only kept</t>
+        </is>
+      </c>
+      <c r="E96" s="12" t="inlineStr">
+        <is>
+          <t>Tab leads straight into a stat grid with no face; badge style inconsistent with the rest of the redesign</t>
+        </is>
+      </c>
+      <c r="F96" s="13" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="G96" s="14" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H96" s="12" t="inlineStr">
+        <is>
+          <t>client-overview/tabs/ProfileInfoTab.tsx</t>
+        </is>
+      </c>
+      <c r="I96" s="12" t="inlineStr">
+        <is>
+          <t>CRM contact records</t>
+        </is>
+      </c>
+      <c r="J96" s="24" t="inlineStr">
+        <is>
+          <t>Spec + mock ready - docs/PF-Profile-Tab-Redesign-Spec.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
board: client dashboard (CL2) + nutrition this-week (NU9) redesign specs; log master-column fix (CO9)
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -946,7 +946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J96"/>
+  <dimension ref="A1:J99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5720,6 +5720,162 @@
       <c r="J96" s="24" t="inlineStr">
         <is>
           <t>Spec + mock ready - docs/PF-Profile-Tab-Redesign-Spec.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="11" t="inlineStr">
+        <is>
+          <t>CL2</t>
+        </is>
+      </c>
+      <c r="B97" s="12" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C97" s="12" t="inlineStr">
+        <is>
+          <t>Client dashboard (NewClientOverview)</t>
+        </is>
+      </c>
+      <c r="D97" s="12" t="inlineStr">
+        <is>
+          <t>Visual polish to coach-grade language: drop gradient bg for flat surface; add CC1 glance-card row; emerald rail on Todays Workout hero; MacroDistributionRibbon on nutrition target card; rounded status pills; demoted Account group. IA from CL1 unchanged</t>
+        </is>
+      </c>
+      <c r="E97" s="12" t="inlineStr">
+        <is>
+          <t>Dashboard still uses gradient bg + generic border cards; reads as a different product from coach surfaces + the shipped Nutrition tab</t>
+        </is>
+      </c>
+      <c r="F97" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G97" s="14" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H97" s="12" t="inlineStr">
+        <is>
+          <t>client/ClientDashboardLayout.tsx, client/NewClientOverview.tsx + composed cards</t>
+        </is>
+      </c>
+      <c r="I97" s="12" t="inlineStr">
+        <is>
+          <t>Coach Overview/Nutrition (own); Runna/Caliber home</t>
+        </is>
+      </c>
+      <c r="J97" s="24" t="inlineStr">
+        <is>
+          <t>Spec + mock ready - docs/CL2-Client-Dashboard-Polish-Spec.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="11" t="inlineStr">
+        <is>
+          <t>NU9</t>
+        </is>
+      </c>
+      <c r="B98" s="12" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C98" s="12" t="inlineStr">
+        <is>
+          <t>Client nutrition This-week form (ClientNutritionProgress)</t>
+        </is>
+      </c>
+      <c r="D98" s="12" t="inlineStr">
+        <is>
+          <t>Restructure the weekly tracking form into a completion-state card stack (weigh-ins/steps/bodyfat+circumference/weekly check-in) w/ status rails + chips matching ClientWeeklyRibbon; mobile Drawer for the heavy inputs. Keep all writes incl bodyfat dual-write</t>
+        </is>
+      </c>
+      <c r="E98" s="12" t="inlineStr">
+        <is>
+          <t>Only laggard on /nutrition-client: still generic shadcn cards, no completion signalling; heaviest client interaction</t>
+        </is>
+      </c>
+      <c r="F98" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G98" s="14" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H98" s="12" t="inlineStr">
+        <is>
+          <t>nutrition/ClientNutritionProgress.tsx</t>
+        </is>
+      </c>
+      <c r="I98" s="12" t="inlineStr">
+        <is>
+          <t>Coach Nutrition (own); habit trackers</t>
+        </is>
+      </c>
+      <c r="J98" s="24" t="inlineStr">
+        <is>
+          <t>Spec + mock ready - docs/NU9-Client-ThisWeek-Tracking-Redesign-Spec.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="11" t="inlineStr">
+        <is>
+          <t>CO9</t>
+        </is>
+      </c>
+      <c r="B99" s="12" t="inlineStr">
+        <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="C99" s="12" t="inlineStr">
+        <is>
+          <t>My Clients master-detail grid</t>
+        </is>
+      </c>
+      <c r="D99" s="12" t="inlineStr">
+        <is>
+          <t>Collapse the master COLUMN width (340px to 220px) when a client is open, not just the card content -- the point of collapsing is to hand the freed width to the detail pane. Smooth grid-template-columns transition</t>
+        </is>
+      </c>
+      <c r="E99" s="12" t="inlineStr">
+        <is>
+          <t>Polish batch condensed the card content but kept the 340px column, so the detail pane gained no room (Hasan caught live)</t>
+        </is>
+      </c>
+      <c r="F99" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G99" s="14" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H99" s="12" t="inlineStr">
+        <is>
+          <t>coach/CoachClientsWorkspace.tsx:351</t>
+        </is>
+      </c>
+      <c r="I99" s="12" t="inlineStr">
+        <is>
+          <t>TrueCoach/Linear master-detail</t>
+        </is>
+      </c>
+      <c r="J99" s="24" t="inlineStr">
+        <is>
+          <t>Shipped (commit ad62f40); pending Vercel deploy + post-deploy smoke</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
board: CL3 client-dashboard polish increment 1 shipped (a9b7fa6); fix CL2 id collision
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -5726,7 +5726,7 @@
     <row r="97">
       <c r="A97" s="11" t="inlineStr">
         <is>
-          <t>CL2</t>
+          <t>CL3</t>
         </is>
       </c>
       <c r="B97" s="12" t="inlineStr">
@@ -5771,7 +5771,7 @@
       </c>
       <c r="J97" s="24" t="inlineStr">
         <is>
-          <t>Spec + mock ready - docs/CL2-Client-Dashboard-Polish-Spec.md</t>
+          <t>Increment 1 SHIPPED (commit a9b7fa6): flat surfaces (drop gradients) + macro ribbon on daily targets. Remaining: optional glance row + status-pill pass. Spec docs/CL2-Client-Dashboard-Polish-Spec.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(rls): relationship-based coach SELECT on weight_logs + circumference_logs; board BUG10
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -946,7 +946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J99"/>
+  <dimension ref="A1:J100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5876,6 +5876,58 @@
       <c r="J99" s="24" t="inlineStr">
         <is>
           <t>Shipped (commit ad62f40); pending Vercel deploy + post-deploy smoke</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="11" t="inlineStr">
+        <is>
+          <t>BUG10</t>
+        </is>
+      </c>
+      <c r="B100" s="12" t="inlineStr">
+        <is>
+          <t>Bug fix</t>
+        </is>
+      </c>
+      <c r="C100" s="12" t="inlineStr">
+        <is>
+          <t>Coach client detail: Progress/Overview/Nutrition</t>
+        </is>
+      </c>
+      <c r="D100" s="12" t="inlineStr">
+        <is>
+          <t>Coach saw "No measurements available" despite client weigh-ins existing. Root cause: weight_logs/circumference_logs coach SELECT keyed on nutrition_phases.coach_id (NULL on seeded phase + stale after reassignment). Fix: relationship-based policy via is_care_team_member_for_client, mirroring body_fat_logs</t>
+        </is>
+      </c>
+      <c r="E100" s="12" t="inlineStr">
+        <is>
+          <t>Coach progress surfaces were empty even with logged data -- silently useless for any client whose phase.coach_id is NULL/stale</t>
+        </is>
+      </c>
+      <c r="F100" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G100" s="14" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H100" s="12" t="inlineStr">
+        <is>
+          <t>migration 20260624140000; weight_logs + circumference_logs RLS</t>
+        </is>
+      </c>
+      <c r="I100" s="12" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J100" s="24" t="inlineStr">
+        <is>
+          <t>SHIPPED + LIVE-VERIFIED 2026-06-24 (applied out-of-band; coach now sees 9 weigh-ins, -1.0kg, chart). Migration file pending commit + db push register</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
board: BUG11 weigh-in week-count alignment shipped + verified (459befe)
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -946,7 +946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J100"/>
+  <dimension ref="A1:J101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5928,6 +5928,58 @@
       <c r="J100" s="24" t="inlineStr">
         <is>
           <t>SHIPPED + LIVE-VERIFIED 2026-06-24 (applied out-of-band; coach now sees 9 weigh-ins, -1.0kg, chart). Migration file pending commit + db push register</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="11" t="inlineStr">
+        <is>
+          <t>BUG11</t>
+        </is>
+      </c>
+      <c r="B101" s="12" t="inlineStr">
+        <is>
+          <t>Bug fix</t>
+        </is>
+      </c>
+      <c r="C101" s="12" t="inlineStr">
+        <is>
+          <t>Client nutrition (/nutrition-client)</t>
+        </is>
+      </c>
+      <c r="D101" s="12" t="inlineStr">
+        <is>
+          <t>Weigh-in count disagreed on the same page: top ribbon showed 1/3 (IGU calendar week) while the new This-week anchor + check-in save-gate showed 0/3 (phase-week). Aligned ClientNutritionProgress anchor + save-gate + N-more notice to startOfIguWeek, matching ribbon + dashboard</t>
+        </is>
+      </c>
+      <c r="E101" s="12" t="inlineStr">
+        <is>
+          <t>User sees two different weigh-in counts seconds apart; save button gated on a different number than displayed</t>
+        </is>
+      </c>
+      <c r="F101" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G101" s="14" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H101" s="12" t="inlineStr">
+        <is>
+          <t>nutrition/ClientNutritionProgress.tsx</t>
+        </is>
+      </c>
+      <c r="I101" s="12" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J101" s="24" t="inlineStr">
+        <is>
+          <t>SHIPPED + LIVE-VERIFIED 2026-06-25 (459befe): anchor now reads 1/3 in agreement with the ribbon</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
board: client sweep CL6-CL9 + WK11 calendar (all live-verified)
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -946,7 +946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J101"/>
+  <dimension ref="A1:J106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5980,6 +5980,266 @@
       <c r="J101" s="24" t="inlineStr">
         <is>
           <t>SHIPPED + LIVE-VERIFIED 2026-06-25 (459befe): anchor now reads 1/3 in agreement with the ribbon</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="11" t="inlineStr">
+        <is>
+          <t>CL6</t>
+        </is>
+      </c>
+      <c r="B102" s="12" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C102" s="12" t="inlineStr">
+        <is>
+          <t>Client dashboard (NewClientOverview)</t>
+        </is>
+      </c>
+      <c r="D102" s="12" t="inlineStr">
+        <is>
+          <t>Desktop: pair right-sized cards 2-col (Daily Targets + Log Today, Weekly Progress + Adherence, Coach + Care Team) instead of full-width stacking. Banners/hero stay full width; mobile stays stacked</t>
+        </is>
+      </c>
+      <c r="E102" s="12" t="inlineStr">
+        <is>
+          <t>Cards stacked full-width even when small (e.g. Log Today = 2 inputs) -- wasted space, poor scan on desktop</t>
+        </is>
+      </c>
+      <c r="F102" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G102" s="14" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H102" s="12" t="inlineStr">
+        <is>
+          <t>client/NewClientOverview.tsx</t>
+        </is>
+      </c>
+      <c r="I102" s="12" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J102" s="24" t="inlineStr">
+        <is>
+          <t>SHIPPED + LIVE-VERIFIED 2026-06-25 (fc77900): Targets+Log side by side confirmed live</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="11" t="inlineStr">
+        <is>
+          <t>CL7</t>
+        </is>
+      </c>
+      <c r="B103" s="12" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C103" s="12" t="inlineStr">
+        <is>
+          <t>Standalone client pages (nutrition, calendar, team-nutrition)</t>
+        </is>
+      </c>
+      <c r="D103" s="12" t="inlineStr">
+        <is>
+          <t>New ClientPageLayout shell (SidebarProvider + ClientSidebar + flat bg). Wrapped ClientNutrition + TeamNutrition so the left nav persists + gradient dropped. WorkoutCalendar gets it via WK10</t>
+        </is>
+      </c>
+      <c r="E103" s="12" t="inlineStr">
+        <is>
+          <t>Sub-pages rendered bare -- left sidebar disappeared + still had the old gradient bg (inconsistent w/ flat dashboard). Hasan flagged it repeated across sub-pages</t>
+        </is>
+      </c>
+      <c r="F103" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G103" s="14" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H103" s="12" t="inlineStr">
+        <is>
+          <t>components/layouts/ClientPageLayout.tsx (new); pages/ClientNutrition.tsx; pages/TeamNutrition.tsx</t>
+        </is>
+      </c>
+      <c r="I103" s="12" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J103" s="24" t="inlineStr">
+        <is>
+          <t>SHIPPED + LIVE-VERIFIED 2026-06-25 (9937518): nutrition page now has left sidebar + flat bg</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="11" t="inlineStr">
+        <is>
+          <t>CL8</t>
+        </is>
+      </c>
+      <c r="B104" s="12" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C104" s="12" t="inlineStr">
+        <is>
+          <t>Dashboard Your Coach card (CoachCard)</t>
+        </is>
+      </c>
+      <c r="D104" s="12" t="inlineStr">
+        <is>
+          <t>Surface the WhatsApp contact-coach button on the dashboard (was only wired into the post-workout completion sheet). Green Message on WhatsApp button w/ the real WhatsApp glyph, gated on coach having a number, via get_coach_whatsapp_for_client RPC; stopPropagation so it does not trigger the cards profile-nav</t>
+        </is>
+      </c>
+      <c r="E104" s="12" t="inlineStr">
+        <is>
+          <t>Built WhatsApp contact feature was invisible to clients on the dashboard; Hasan asked where it was + wanted the real WA logo</t>
+        </is>
+      </c>
+      <c r="F104" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G104" s="14" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H104" s="12" t="inlineStr">
+        <is>
+          <t>client/CoachCard.tsx</t>
+        </is>
+      </c>
+      <c r="I104" s="12" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J104" s="24" t="inlineStr">
+        <is>
+          <t>SHIPPED + LIVE-VERIFIED 2026-06-25 (550c964): green WhatsApp button renders on Your Coach card</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="11" t="inlineStr">
+        <is>
+          <t>CL9</t>
+        </is>
+      </c>
+      <c r="B105" s="12" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C105" s="12" t="inlineStr">
+        <is>
+          <t>Client nutrition page (/nutrition-client)</t>
+        </is>
+      </c>
+      <c r="D105" s="12" t="inlineStr">
+        <is>
+          <t>Regroup desktop layout: Row A = target/calorie phase card beside the trend graph; Row B = weekly ribbon + daily log paired; This-week form full width. lg breakpoint (sidebar eats width on md)</t>
+        </is>
+      </c>
+      <c r="E105" s="12" t="inlineStr">
+        <is>
+          <t>Cards stacked full-width single column -- oversized for content, related info (target + graph) not grouped. Hasan flagged grouping + sizing</t>
+        </is>
+      </c>
+      <c r="F105" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G105" s="14" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H105" s="12" t="inlineStr">
+        <is>
+          <t>pages/ClientNutrition.tsx</t>
+        </is>
+      </c>
+      <c r="I105" s="12" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J105" s="24" t="inlineStr">
+        <is>
+          <t>SHIPPED + LIVE-VERIFIED 2026-06-25 (3fcf6dd): phase card beside graph, not cramped; ribbon+log paired</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="11" t="inlineStr">
+        <is>
+          <t>WK11</t>
+        </is>
+      </c>
+      <c r="B106" s="12" t="inlineStr">
+        <is>
+          <t>Workout</t>
+        </is>
+      </c>
+      <c r="C106" s="12" t="inlineStr">
+        <is>
+          <t>Client workout calendar (/client/workout/calendar)</t>
+        </is>
+      </c>
+      <c r="D106" s="12" t="inlineStr">
+        <is>
+          <t>Rebuilt the bare month-grid-with-dots into a WK10 week-grid: 7 day columns w/ color-coded session chips (title + completed/scheduled), week nav + This-week jump, today highlighted, in the ClientPageLayout shell. Mobile = Runna-style day list. useClientWorkoutsWeek extended w/ title+date</t>
+        </is>
+      </c>
+      <c r="E106" s="12" t="inlineStr">
+        <is>
+          <t>Calendar opened standalone (no left nav) + looked nothing like the WK10 design we built (was month dots). Hasan flagged both</t>
+        </is>
+      </c>
+      <c r="F106" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G106" s="14" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H106" s="12" t="inlineStr">
+        <is>
+          <t>pages/client/WorkoutCalendar.tsx (rewrite); hooks/useClientWorkouts.ts</t>
+        </is>
+      </c>
+      <c r="I106" s="12" t="inlineStr">
+        <is>
+          <t>TrueCoach week calendar; Runna day list</t>
+        </is>
+      </c>
+      <c r="J106" s="24" t="inlineStr">
+        <is>
+          <t>SHIPPED + LIVE-VERIFIED 2026-06-25 (7608f0c) desktop + mobile; seeded a test program to confirm chips render</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
board: client sweep + recomposition (CL6 main+rail, CL7 shell pages, CL8 WhatsApp, CL9 nutrition, WK11 calendar)
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -6001,7 +6001,7 @@
       </c>
       <c r="D102" s="12" t="inlineStr">
         <is>
-          <t>Desktop: pair right-sized cards 2-col (Daily Targets + Log Today, Weekly Progress + Adherence, Coach + Care Team) instead of full-width stacking. Banners/hero stay full width; mobile stays stacked</t>
+          <t>Recompose dashboard into MAIN + RAIL: full-width Today hero on top; main column = nutrition target / this-week / adherence; rail = log today / coach (WhatsApp) / care team. Columns flow independently so short rail cards fill height vs a taller main -- no dead space. Replaces the forced equal-2col pairs</t>
         </is>
       </c>
       <c r="E102" s="12" t="inlineStr">
@@ -6031,7 +6031,7 @@
       </c>
       <c r="J102" s="24" t="inlineStr">
         <is>
-          <t>SHIPPED + LIVE-VERIFIED 2026-06-25 (fc77900): Targets+Log side by side confirmed live</t>
+          <t>SHIPPED + LIVE-VERIFIED 2026-06-25 desktop+mobile (609a9e9; earlier 2col fc77900). Balanced, important-first, grouped per Hasan geometry/flow note</t>
         </is>
       </c>
     </row>
@@ -6083,7 +6083,7 @@
       </c>
       <c r="J103" s="24" t="inlineStr">
         <is>
-          <t>SHIPPED + LIVE-VERIFIED 2026-06-25 (9937518): nutrition page now has left sidebar + flat bg</t>
+          <t>SHIPPED + LIVE-VERIFIED 2026-06-25 (9937518 + bd66f70): ClientPageLayout shell wraps ClientNutrition, TeamNutrition, WorkoutCalendar, Messages, ExerciseHistory, AddonsCatalog. REMAINING: ClientSessions (4 returns) + shared multi-role Account/WorkoutLibrary/EducationalVideos (need role-aware layout)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Merge Exercise Library + Videos + Pathways into unified /learn area
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -946,7 +946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J106"/>
+  <dimension ref="A1:J110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6083,7 +6083,7 @@
       </c>
       <c r="J103" s="24" t="inlineStr">
         <is>
-          <t>SHIPPED + LIVE-VERIFIED 2026-06-25 (9937518 + bd66f70): ClientPageLayout shell wraps ClientNutrition, TeamNutrition, WorkoutCalendar, Messages, ExerciseHistory, AddonsCatalog. REMAINING: ClientSessions (4 returns) + shared multi-role Account/WorkoutLibrary/EducationalVideos (need role-aware layout)</t>
+          <t>SHIPPED + LIVE-VERIFIED 2026-06-25 (9937518 + bd66f70): ClientPageLayout shell wraps ClientNutrition, TeamNutrition, WorkoutCalendar, Messages, ExerciseHistory, AddonsCatalog. REMAINING: ClientSessions (4 returns) + shared multi-role Account/WorkoutLibrary/EducationalVideos (need role-aware layout)  [UPDATE 2026-06-25: REMAINING done by CL10 -- ClientPageLayout now role-aware + wraps ClientSessions/Account/Learn.]</t>
         </is>
       </c>
     </row>
@@ -6240,6 +6240,214 @@
       <c r="J106" s="24" t="inlineStr">
         <is>
           <t>SHIPPED + LIVE-VERIFIED 2026-06-25 (7608f0c) desktop + mobile; seeded a test program to confirm chips render</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>NU10</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Nutrition</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Weekly check-in (ClientNutritionProgress)</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Unify the whole weekly check-in into ONE guided surface: 3-level adherence scale (on_point/mostly/off_track + weighed/estimated/guessed) replacing yes/no; grouped Adherence + How-you-feel (changes + note) + cadence-gated Measurements (weight always; circumference odd weeks; body fat every 4th) with Steps folded in; dimmed dietitian-scoped Advanced seam. Persists note + physical_changes on adherence_logs.</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Scattered adherence+changes across cards; richer signal; one phase-scoped write; extensible to dietitian questions.</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>nutrition/ClientNutritionProgress.tsx; nutrition/NutritionProgress.tsx; supabase/migrations 20260625120000 + 20260625130000; integrations/supabase/types.ts</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>visualize mock client_unified_checkin</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>SHIPPED + LIVE-VERIFIED 2026-06-25 (a55d9b6 + 5f681a0 + 8144fb0): 3-level scale + derived compat booleans (lenient: mostly/estimated=true) so coach roster % math unchanged; steps fold-in; notes+physical_changes on adherence_logs. Caught + fixed pre-existing weekly_progress.goal_id FK landmine (nutrition_phases vs nutrition_goals disjoint) that 409d notes/body-fat for ALL phase clients -- check-in no longer writes weekly_progress; body fat relies on body_fat_logs. Supersedes NU9.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>CT5</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Library (Learn)</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Merge Exercise Library + Educational Videos + Learning Paths into one /learn area: segmented Exercises . Videos . Pathways over a shared search; Exercises keeps full taxonomy facets; admin keeps video CMS in Videos tab; coach gets preview + assign. Old routes redirect; all nav repointed.</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Three fragmented content surfaces; stop spreading features -- unify+simplify (Mobbin: NTC/MasterClass/Headspace single library + segmented tabs).</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>pages/Learn.tsx (new); components/learn/ExercisesTab.tsx + VideosTab.tsx (new); lib/routeConfig.ts; client/ClientSidebar.tsx; Navigation.tsx; client/QuickActionsGrid.tsx; App.tsx</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Nike Training Club / MasterClass / Headspace</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>BUILT 2026-06-25, tsc-clean; PENDING push + live-verify. /workout-library -&gt; /learn?tab=exercises and /educational-videos -&gt; /learn?tab=videos redirect; sidebar/mobile-dock/top-nav/quick-action all repoint to Learn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>WK12</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Workout</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Workouts area (/client/workout/calendar)</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Rename calendar -&gt; Workouts; Schedule/History in-page tabs (fold Exercise History in, remove its separate nav item); Week/Month toggle (default Month); month grid w/ status dots + legend + This-week enriched brief list (exercise count + primary muscles + Done/Due/Scheduled/Missed rails); enriched week chips; Message-coach button (-&gt; /messages); tap a month day to jump to that week.</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Calendar was a bare week-grid; enrich + unify; month view is denser (Hasan pref); brief = exercise count + primary muscles.</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>pages/client/WorkoutCalendar.tsx (rewrite); components/workouts/ExerciseHistoryPanel.tsx (new); hooks/useClientWorkouts.ts (enriched month/week selects + deriveModuleBrief); lib/routeConfig.ts; client/ClientSidebar.tsx; Navigation.tsx; App.tsx</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Runna / Nike Training Club</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>BUILT 2026-06-25, tsc-clean; PENDING push + live-verify. Exercise History folded into Workouts&gt;History tab; /client/workout/history redirects to ?tab=history; nav item removed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>CL10</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Role-aware ClientPageLayout + audit tail</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Make ClientPageLayout ROLE-AWARE (client -&gt; full sidebar shell; coach/admin -&gt; bare, top-nav only w/ correct role) via warm useRoleCache + fallback user_roles fetch. Wrap Learn, AccountManagement (2 branches), ClientSessions (4 branches) so staff stop getting the client sidebar / forced client role on shared multi-role routes.</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Completes CL7: shared multi-role pages either lost the nav (bare) or would force the client shell on coaches/admins.</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>components/layouts/ClientPageLayout.tsx; pages/Learn.tsx; pages/AccountManagement.tsx; pages/ClientSessions.tsx</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>BUILT 2026-06-25, tsc-clean; PENDING push + live-verify incl. coach-login check on a shared page. Closes the CL7 REMAINING item (ClientSessions + role-aware shell for Account/Learn).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Board: mark Learn/Workouts/role-aware shell live-verified
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -6343,7 +6343,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>BUILT 2026-06-25, tsc-clean; PENDING push + live-verify. /workout-library -&gt; /learn?tab=exercises and /educational-videos -&gt; /learn?tab=videos redirect; sidebar/mobile-dock/top-nav/quick-action all repoint to Learn.</t>
+          <t>SHIPPED + LIVE-VERIFIED 2026-06-25 (57321da) desktop+mobile: segmented Exercises/Videos/Pathways + shared search + full taxonomy facets; /workout-library and /educational-videos redirect into /learn; mobile dock shows Learn. Admin video-CMS + coach assign branches preserved.</t>
         </is>
       </c>
     </row>
@@ -6395,7 +6395,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>BUILT 2026-06-25, tsc-clean; PENDING push + live-verify. Exercise History folded into Workouts&gt;History tab; /client/workout/history redirects to ?tab=history; nav item removed.</t>
+          <t>SHIPPED + LIVE-VERIFIED 2026-06-25 (57321da) desktop+mobile: Schedule/History tabs, Month default w/ status dots+legend + This-week briefs (status rails/pills), Week toggle enriched chips (count + status), folded ExerciseHistory panel, Message-coach, /client/workout/history redirect, dock renamed Workouts. (Seeded test program has 0 module_exercises so briefs show 0 exercises/no muscles -- count logic correct; real programs populate muscles.)</t>
         </is>
       </c>
     </row>
@@ -6447,7 +6447,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>BUILT 2026-06-25, tsc-clean; PENDING push + live-verify incl. coach-login check on a shared page. Closes the CL7 REMAINING item (ClientSessions + role-aware shell for Account/Learn).</t>
+          <t>SHIPPED + LIVE-VERIFIED (client side) 2026-06-25 (57321da): client gets the sidebar shell on Learn/Workouts/Account; Account shows only the Account tab (no Coach Profile) for a client. PENDING: coach-login pass to confirm staff get the BARE shell (no client sidebar) on a shared route.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Board: log CT6 Coach Hub, CO10 collapsible client list, CO11 coach design polish
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -946,7 +946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J110"/>
+  <dimension ref="A1:J113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6448,6 +6448,162 @@
       <c r="J110" t="inlineStr">
         <is>
           <t>SHIPPED + LIVE-VERIFIED (client side) 2026-06-25 (57321da): client gets the sidebar shell on Learn/Workouts/Account; Account shows only the Account tab (no Coach Profile) for a client. PENDING: coach-login pass to confirm staff get the BARE shell (no client sidebar) on a shared route.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>CT6</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Coach Hub (/coach/hub)</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>New coach-only education area: segmented Training / Library / Resources over shared search. Library = advanced coach-only videos (category+level filters); Resources = ebooks/links + courses/certifications (redirect out). Generalized coach_educational_content (content_type/section/category/level/external_url/author); admin CMS extended; training gate scoped to section=training.</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Centralizes advanced coaching education separate from client content; closes an RLS leak where any authenticated user could read coach content.</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>src/pages/coach/CoachHub.tsx; CoachTrainingDashboard.tsx; admin/CoachEducationalContentManager.tsx; routeConfig.ts; App.tsx; migration 20260625140000</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>MasterClass; Crypto.com University</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-06-25 (c7dc303); coach live-verify pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>CO10</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>My Clients workspace (desktop)</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Collapse the master client list to a 48px rail when a client is open so the detail pane gets the full canvas; chevron+clients-icon+attention-dot to expand into the full picker; auto-collapse on select. Desktop only; mobile keeps the drawer.</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Coaches need room to read an individual client’s cards on desktop; the 220px master ate width with no payoff once focused.</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>src/components/coach/CoachClientsWorkspace.tsx</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Linear; Height (master-detail collapse)</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-06-25 (2863664); coach live-verify pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>CO11</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Coach shell + cards (design-language polish)</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Flatten 3 leftover to-primary/5 gradients to bg-background (CoachDashboardLayout, CoachContentAssignments, TeamMemberNutritionDialog); swap macrocycle block &lt;Card onClick&gt; to ClickableCard (keyboard + aria-label).</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Brings coach surfaces in line with the flat-dark design language and a11y card pattern used everywhere else.</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>src/components/coach/CoachDashboardLayout.tsx; CoachContentAssignments.tsx; TeamMemberNutritionDialog.tsx; programs/macrocycles/MacrocycleEditor.tsx</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-06-25 (2863664)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Board: log CO12 retire Progress tab + promote weight trend
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -946,7 +946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J113"/>
+  <dimension ref="A1:J114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6604,6 +6604,58 @@
       <c r="J113" t="inlineStr">
         <is>
           <t>SHIPPED 2026-06-25 (2863664)</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>CO12</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Individual client overview (/coach/clients/:id)</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Retire the redundant Progress tab (its CoachNutritionGraphs already lives in Nutrition-&gt;History; its VolumeChart already lives in Workouts). 8 sections -&gt; 7. Promote a compact phase-scoped weight-trend card onto Nutrition-&gt;Overview so the line is visible without drilling into History. Deep links to ?tab=progress degrade to default via the existing unknown-slug guard.</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Removes a duplicate page; surfaces the weight trend one fewer click away. Simplify + avoid redundant pages.</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>src/components/client-overview/sections.ts; ClientOverviewTabs.tsx; ClientOverviewNav.tsx; tabs/NutritionTab.tsx; nutrition/PhaseWeightTrendCard.tsx (new); tabs/ProgressTab.tsx (deleted)</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Linear; Notion (consolidated detail views)</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-06-25 (39050a3); coach live-verify pending</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Board: log CO13 coach polish pass (sidebar persistence, weight-trend domain, copy, mono numbers)
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -946,7 +946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J114"/>
+  <dimension ref="A1:J115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6656,6 +6656,58 @@
       <c r="J114" t="inlineStr">
         <is>
           <t>SHIPPED 2026-06-25 (39050a3); coach live-verify pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>CO13</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Coach surfaces (polish pass)</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Live-review polish: (1) weight-trend Y-domain now spans start+target so the target line is never off-chart; (2) new CoachShell wraps Coach Hub + Content Assignments so the left sidebar rail persists on those standalone pages; (3) Content Assignments empty-state copy points to Learn (was dead /educational-videos); program with no title falls back to macrocycle name then "Training program" (was "Untitled program"); (4) MetricCard hero value now font-mono+tabular app-wide; team cards equal-height + ClickableCard (was &lt;Card onClick&gt;). Capacity bars left as-is (load-encoded colours are intentional).</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Consistency + discoverability across the coach experience; removes dead copy and a11y/card anti-patterns.</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>PhaseWeightTrendCard.tsx; useClientWorkouts.ts; coach/CoachShell.tsx (new); coach/teams/TeamCard.tsx; ui/metric-card.tsx; pages/coach/CoachHub.tsx; pages/coach/CoachContentAssignments.tsx</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Linear; Height</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>SHIPPED + LIVE-VERIFIED 2026-06-25 (162155f)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Board: log DS1 design foundation (Geist, flat Card, weight ceiling)
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -946,7 +946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J115"/>
+  <dimension ref="A1:J116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6708,6 +6708,58 @@
       <c r="J115" t="inlineStr">
         <is>
           <t>SHIPPED + LIVE-VERIFIED 2026-06-25 (162155f)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>DS1</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Design foundation (typography + card primitive)</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>App-wide foundation pass to close the gap between mockups and the live UI: (1) swap body typeface DM Sans -&gt; Geist (index.html link + tailwind sans token); (2) flatten the Card primitive -- drop shadow-sm so cards sit flat with a hairline border instead of the stock shadcn float; (3) cap font-bold at 600 via tailwind fontWeight theme override (every 700 header -&gt; crisp 600 in one place); (4) CardTitle 600 -&gt; 500. Bebas Neue display headlines + JetBrains Mono numerals unchanged.</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Mockups read more premium than the site due to heavy 700 weights + shadowed stock-shadcn cards + generic font. Foundation-level fix lifts every page (client/coach/public/admin) at once.</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>index.html; tailwind.config.ts; src/components/ui/card.tsx</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Linear; Vercel/Geist; Anthropic design system</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>SHIPPED + LIVE-VERIFIED 2026-06-26 (coach dashboard + client overview + public /services)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Board cleanup: close PR1 (superseded by CO12), verify CO2, resolve CT1+CL3 ID collisions
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -1749,7 +1749,7 @@
       </c>
       <c r="J16" s="28" t="inlineStr">
         <is>
-          <t>Spec ready — small token pass on CoachOverviewStats / activity icons / compensation badges; no fabricated deltas. P2.</t>
+          <t>SHIPPED + LIVE-VERIFIED 2026-06-26 — metric cards carry interpretation/direction lines (e.g. "1 check-in due — 1 is 11d overdue", "7 of 7 clients active"); token pass folded into DS1 (mono numbers, flat cards). No fabricated deltas.</t>
         </is>
       </c>
     </row>
@@ -5615,14 +5615,14 @@
       </c>
       <c r="J94" s="24" t="inlineStr">
         <is>
-          <t>Spec + mock ready - docs/PR-Progress-Tab-Redesign-Spec.md</t>
+          <t>CLOSED 2026-06-26 — SUPERSEDED by CO12: the Progress tab was removed entirely (its CoachNutritionGraphs already lived in Nutrition-&gt;History; VolumeChart in Workouts) and a compact weight trend was promoted onto Nutrition-&gt;Overview. Redesign moot.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="11" t="inlineStr">
         <is>
-          <t>CT1</t>
+          <t>CARE1</t>
         </is>
       </c>
       <c r="B95" s="12" t="inlineStr">
@@ -5667,7 +5667,7 @@
       </c>
       <c r="J95" s="24" t="inlineStr">
         <is>
-          <t>Spec + mock ready - docs/CT-CareTeam-Tab-Redesign-Spec.md</t>
+          <t>Spec + mock ready - docs/CT-CareTeam-Tab-Redesign-Spec.md [ID renamed CT1-&gt;CARE1 2026-06-26 to resolve collision with CT1 Content/Library row 53.]</t>
         </is>
       </c>
     </row>
@@ -5726,7 +5726,7 @@
     <row r="97">
       <c r="A97" s="11" t="inlineStr">
         <is>
-          <t>CL3</t>
+          <t>CL11</t>
         </is>
       </c>
       <c r="B97" s="12" t="inlineStr">
@@ -5771,7 +5771,7 @@
       </c>
       <c r="J97" s="24" t="inlineStr">
         <is>
-          <t>Increment 1 SHIPPED (commit a9b7fa6): flat surfaces (drop gradients) + macro ribbon on daily targets. Remaining: optional glance row + status-pill pass. Spec docs/CL2-Client-Dashboard-Polish-Spec.md</t>
+          <t>Increment 1 SHIPPED (commit a9b7fa6): flat surfaces (drop gradients) + macro ribbon on daily targets. Remaining: optional glance row + status-pill pass. Spec docs/CL2-Client-Dashboard-Polish-Spec.md [ID renamed CL3-&gt;CL11 2026-06-26 to resolve collision with CL3 LogTodayCard row 12.]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: session artifacts — handover + design-board updates + day-move/B6 specs
- HANDOVER.md: rewritten for the next Cowork session (Track 1 P5 Stage A live +
  Stage B gates D3/re-key/soak; Track 2 design backlog triage; open items; refs).
- docs/IGU-Design-Changes-Master.xlsx: HX1 status appended with the 2026-07-04
  e1RM supersession note (NO e1RM — replace the Estimated-1RM trend card with actual
  logged rep-maxes; pending small re-slice); WK13 (day-move) + MS4 (contextual
  comments) rows appended as shipped + live-verified.
- docs/DAY_MOVE_SLICE_BUILD.md + docs/B6_CONTEXTUAL_COMMENTS_BUILD.md: the two
  build specs (T5_TEAM_BACKFILL_BUILD.md already tracked).

Docs only — no code/bundle change.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/IGU-Design-Changes-Master.xlsx
+++ b/docs/IGU-Design-Changes-Master.xlsx
@@ -946,7 +946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J116"/>
+  <dimension ref="A1:J118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2640,7 +2640,7 @@
       </c>
       <c r="J34" s="28" t="inlineStr">
         <is>
-          <t>Shipped — merged main PR #167 (1b5f9c6), deploys to prod via Vercel. ExerciseHistory leads with Estimated-1RM trend MetricCard (Epley via shared helper; sparkline+delta+interpretE1rmTrend gated &gt;=2 sessions) + 3 per-session PR tiles; chronological table kept. Visual confirm at post-deploy smoke.</t>
+          <t>Shipped — merged main PR #167 (1b5f9c6), deploys to prod via Vercel. ExerciseHistory leads with Estimated-1RM trend MetricCard (Epley via shared helper; sparkline+delta+interpretE1rmTrend gated &gt;=2 sessions) + 3 per-session PR tiles; chronological table kept. Visual confirm at post-deploy smoke. || SUPERSEDED IN PART 2026-07-04: Hasan decision = NO e1RM anywhere in the app. Replace the Estimated-1RM trend card with ACTUAL logged rep-maxes (best load per rep count); true 1RM = coach programs a test day. Pending re-slice (small).</t>
         </is>
       </c>
     </row>
@@ -6760,6 +6760,102 @@
       <c r="J116" t="inlineStr">
         <is>
           <t>SHIPPED + LIVE-VERIFIED 2026-06-26 (coach dashboard + client overview + public /services)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>WK13</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Workout</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Program board + coach calendar</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Move session to another day: board kebab 'Move to day' (dated start-anchored picker) + 'apply to following weeks?' cascade prompt + coach-calendar move via move_plan_session RPC (1:1 clones only; team-shared rejected -&gt; 'edit from the team board')</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Coaches adjust a client schedule without rebuilding weeks; the one net-new board affordance from the redesign (B4/B5 tails)</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>MuscleBuilderPage/SessionBlock/MobileDayDetail/ClientScheduleCalendar + move_plan_session RPC</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr"/>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>SHIPPED + LIVE-VERIFIED 2026-07-02 (spec docs/DAY_MOVE_SLICE_BUILD.md). 3 smoke-found anchor-label bugs fixed same day (picker off-by-one, toast copy, mobile day-strip) - LESSON: all board weekday labels derive from assignment-start anchor, never Mon-first. Follow-up (merged 7ee0f02): copy/paste-day + remove-muscle toasts anchored too.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>MS4</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Messaging</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Contextual comments</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Per-object comment threads on a logged session / weekly check-in / nutrition adjustment (coach&lt;-&gt;client two-way), distinct from general chat and care-team messages</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Feedback lives where it's relevant ('great pressing' on THE session); closes the redesign doc's B6 - last increment of COACH_CLIENT_REDESIGN.md</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>contextual_comments table + trigger + ContextualCommentThread; mounts: SessionLogViewer/NutritionCheckInCard/NutritionAdjustmentWeekCard/ClientNutritionProgress</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr"/>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>SHIPPED + LIVE-VERIFIED 2026-07-03/04 (spec docs/B6_CONTEXTUAL_COMMENTS_BUILD.md; migration 20260703120000). RLS matrix + ownership trigger DB-proven; two-way check-in thread live; author names via get_coach_for_client (NOT coaches_client_safe - RLS-broken for clients). REMAINING fast-follows: client-side session+adjustment threads (no host surface yet), unread badges/notifications.</t>
         </is>
       </c>
     </row>

</xml_diff>